<commit_message>
Add JL-2 third stage with calculated burn times
Stage 3 sized relative to stages 1 & 2: propellant follows the geometric
mass taper (P2/P1 ~ 0.56) -> 7.39 t, tapered to 1.8 m diameter (0.9x),
giving a 2.11 m motor. The 4.32 m shroud then leaves a 2.21 m warhead bay
(out of scope; RV mass not carried in the stack).

Burn times are now CALCULATED for all stages from the P35 mass-flow anchor
(35 t / 71 s = 493 kg/s at 2.0 m; throat area ~ diameter^2), replacing the
earlier placeholders:
  S1  47.2 s, 1315 kN vac   S2  26.6 s, 1315 kN   S3  18.5 s, 1065 kN
This reproduces P35's quoted ~1176 kN thrust and gives a 2.46 liftoff T/W.

Per-stage mass_initial now chains all three motors (49.7 t wet stack).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FYmY1XBusSrATRZ4jAxiDg
</commit_message>
<xml_diff>
--- a/models/JL-2.xlsx
+++ b/models/JL-2.xlsx
@@ -645,12 +645,14 @@
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>41318</v>
+        <v>49718</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>14897</v>
-      </c>
-      <c r="F7" s="4" t="n"/>
+        <v>23297</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>8400</v>
+      </c>
       <c r="G7" s="4" t="n"/>
       <c r="I7" s="5" t="inlineStr">
         <is>
@@ -675,7 +677,9 @@
       <c r="E8" s="4" t="n">
         <v>13110</v>
       </c>
-      <c r="F8" s="4" t="n"/>
+      <c r="F8" s="4" t="n">
+        <v>7392</v>
+      </c>
       <c r="G8" s="4" t="n"/>
       <c r="I8" s="5" t="inlineStr"/>
     </row>
@@ -696,7 +700,9 @@
       <c r="E9" s="4" t="n">
         <v>1788</v>
       </c>
-      <c r="F9" s="4" t="n"/>
+      <c r="F9" s="4" t="n">
+        <v>1008</v>
+      </c>
       <c r="G9" s="4" t="n"/>
       <c r="I9" s="5" t="inlineStr">
         <is>
@@ -721,7 +727,9 @@
       <c r="E10" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="4" t="n"/>
+      <c r="F10" s="4" t="n">
+        <v>1.8</v>
+      </c>
       <c r="G10" s="4" t="n"/>
       <c r="I10" s="5" t="inlineStr"/>
     </row>
@@ -742,7 +750,9 @@
       <c r="E11" s="4" t="n">
         <v>2.94</v>
       </c>
-      <c r="F11" s="4" t="n"/>
+      <c r="F11" s="4" t="n">
+        <v>2.11</v>
+      </c>
       <c r="G11" s="4" t="n"/>
       <c r="I11" s="5" t="inlineStr"/>
     </row>
@@ -758,12 +768,14 @@
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>1292033</v>
+        <v>1314920</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>728514</v>
-      </c>
-      <c r="F12" s="4" t="n"/>
+        <v>1314920</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>1065085</v>
+      </c>
       <c r="G12" s="4" t="n"/>
       <c r="I12" s="5" t="inlineStr">
         <is>
@@ -783,12 +795,14 @@
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>48</v>
+        <v>47.1645505490343</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>48</v>
-      </c>
-      <c r="F13" s="4" t="n"/>
+        <v>26.59377608725181</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>18.51225383079049</v>
+      </c>
       <c r="G13" s="4" t="n"/>
       <c r="I13" s="5" t="inlineStr"/>
     </row>
@@ -809,7 +823,9 @@
       <c r="E14" s="4" t="n">
         <v>272</v>
       </c>
-      <c r="F14" s="4" t="n"/>
+      <c r="F14" s="4" t="n">
+        <v>272</v>
+      </c>
       <c r="G14" s="4" t="n"/>
       <c r="I14" s="5" t="inlineStr">
         <is>
@@ -829,12 +845,14 @@
         </is>
       </c>
       <c r="D15" s="4" t="n">
-        <v>1.13</v>
+        <v>1.15</v>
       </c>
       <c r="E15" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="4" t="n"/>
+      <c r="F15" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="G15" s="4" t="n"/>
       <c r="I15" s="5" t="inlineStr">
         <is>
@@ -865,7 +883,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -917,7 +935,9 @@
       <c r="E18" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F18" s="4" t="n"/>
+      <c r="F18" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="G18" s="4" t="n"/>
       <c r="I18" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add hydrodynamic fairing to JL-2 model, jettisoned at 2 km
The 608 px (4.32 m) forward shroud is a water-egress structure, not an
atmospheric fairing: it sheds seconds into flight (2 km jettison altitude)
rather than the 80 km launch-vehicle default.

Mass ~298 kg from the Akin fairing MER (mass_estimator.fairing_mass) with
a 1.5x hydrodynamic-loads factor on the 24.8 m2 wetted area; blunt parabola
nose profile, 1.5 m nose length. Carried on stage 1 only; launch mass is
now 50.0 t (motors + fairing, no warhead).

Detailed workbook only — the catalog draft format has no shroud columns.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FYmY1XBusSrATRZ4jAxiDg
</commit_message>
<xml_diff>
--- a/models/JL-2.xlsx
+++ b/models/JL-2.xlsx
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>49718</v>
+        <v>50016</v>
       </c>
       <c r="E7" s="4" t="n">
         <v>23297</v>
@@ -1618,7 +1618,7 @@
         </is>
       </c>
       <c r="D60" s="4" t="n">
-        <v>0</v>
+        <v>298</v>
       </c>
       <c r="I60" s="5" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         </is>
       </c>
       <c r="D61" s="4" t="n">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="I61" s="5" t="inlineStr">
         <is>
@@ -1658,7 +1658,7 @@
         </is>
       </c>
       <c r="D62" s="4" t="n">
-        <v>0</v>
+        <v>4.32</v>
       </c>
       <c r="I62" s="5" t="inlineStr"/>
     </row>
@@ -1674,7 +1674,7 @@
         </is>
       </c>
       <c r="D63" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I63" s="5" t="inlineStr"/>
     </row>
@@ -1689,7 +1689,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D64" s="4" t="inlineStr"/>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>Parabola</t>
+        </is>
+      </c>
       <c r="I64" s="5" t="inlineStr"/>
     </row>
     <row r="65">
@@ -1704,7 +1708,7 @@
         </is>
       </c>
       <c r="D65" s="4" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I65" s="5" t="inlineStr"/>
     </row>

</xml_diff>